<commit_message>
adiciona rotulação dos dados de teste
</commit_message>
<xml_diff>
--- a/resultados/test1_rotulado.xlsx
+++ b/resultados/test1_rotulado.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3892,7 +3892,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5164,7 +5164,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5404,7 +5404,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5476,7 +5476,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5908,7 +5908,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -5956,7 +5956,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6256,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -6532,7 +6532,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6772,7 +6772,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7060,7 +7060,7 @@
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -7420,7 +7420,7 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -7564,7 +7564,7 @@
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7864,7 @@
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8056,7 +8056,7 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8104,7 @@
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -8452,7 +8452,7 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8560,7 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8836,7 +8836,7 @@
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9244,7 +9244,7 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -9256,7 +9256,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9304,7 +9304,7 @@
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9352,7 +9352,7 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9592,7 @@
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10000,7 +10000,7 @@
       </c>
       <c r="B798" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10024,7 +10024,7 @@
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10036,7 +10036,7 @@
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10240,7 +10240,7 @@
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10396,7 +10396,7 @@
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10504,7 +10504,7 @@
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10588,7 +10588,7 @@
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>c5</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10600,7 +10600,7 @@
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -10720,7 +10720,7 @@
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10732,7 @@
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>c234</t>
+          <t>c1</t>
         </is>
       </c>
     </row>
@@ -10948,7 +10948,7 @@
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c5</t>
         </is>
       </c>
     </row>
@@ -11092,7 +11092,7 @@
       </c>
       <c r="B889" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>
@@ -11224,7 +11224,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>c1</t>
+          <t>c234</t>
         </is>
       </c>
     </row>

</xml_diff>